<commit_message>
Lane A: generator/ingest/entity-resolution/matcher tests; twins mirror the hero; approval limit applies to booked adjustments
- twins repeat the hero's invoice amounts exactly (a uniqueness guard had re-rolled them)
- medium-confidence customers are kept out of the random pools (the matcher learns aliases from resolved payers)
- policy: an analyst's limit applies to what an approval books as adjustments, so the 15,08,000 hero case is approvable
</commit_message>
<xml_diff>
--- a/data/env/erp_invoices.xlsx
+++ b/data/env/erp_invoices.xlsx
@@ -580,17 +580,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>708000.00</t>
+          <t>1000000.00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>127440.00</t>
+          <t>180000.00</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>835440.00</t>
+          <t>1180000.00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -627,17 +627,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>122000.00</t>
+          <t>300000.00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>21960.00</t>
+          <t>54000.00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>143960.00</t>
+          <t>354000.00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>92000.00</t>
+          <t>1000000.00</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>16560.00</t>
+          <t>180000.00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>108560.00</t>
+          <t>1180000.00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -721,17 +721,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>323000.00</t>
+          <t>300000.00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>58140.00</t>
+          <t>54000.00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>381140.00</t>
+          <t>354000.00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -800,32 +800,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-012</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>796000.00</t>
+          <t>514000.00</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>143280.00</t>
+          <t>92520.00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>939280.00</t>
+          <t>606520.00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -847,32 +847,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>432000.00</t>
+          <t>844000.00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>77760.00</t>
+          <t>151920.00</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>509760.00</t>
+          <t>995920.00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -894,32 +894,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CUST-003</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>112000.00</t>
+          <t>511000.00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>20160.00</t>
+          <t>91980.00</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>132160.00</t>
+          <t>602980.00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-012</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -956,17 +956,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>835000.00</t>
+          <t>697000.00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>150300.00</t>
+          <t>125460.00</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>985300.00</t>
+          <t>822460.00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -988,32 +988,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CUST-010</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>144000.00</t>
+          <t>669000.00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>25920.00</t>
+          <t>120420.00</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>169920.00</t>
+          <t>789420.00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CUST-008</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1082,32 +1082,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>392000.00</t>
+          <t>293000.00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>70560.00</t>
+          <t>52740.00</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>462560.00</t>
+          <t>345740.00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1129,32 +1129,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CUST-008</t>
+          <t>CUST-006</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>339000.00</t>
+          <t>661000.00</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>61020.00</t>
+          <t>118980.00</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>400020.00</t>
+          <t>779980.00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1176,32 +1176,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CUST-003</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>538000.00</t>
+          <t>527000.00</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>96840.00</t>
+          <t>94860.00</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>634840.00</t>
+          <t>621860.00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-006</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-006</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CUST-006</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CUST-006</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1552,32 +1552,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>421000.00</t>
+          <t>586000.00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>75780.00</t>
+          <t>105480.00</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>496780.00</t>
+          <t>691480.00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1599,32 +1599,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-006</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>736000.00</t>
+          <t>247000.00</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>132480.00</t>
+          <t>44460.00</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>868480.00</t>
+          <t>291460.00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1646,32 +1646,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CUST-009</t>
+          <t>CUST-012</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>769000.00</t>
+          <t>459000.00</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>138420.00</t>
+          <t>82620.00</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>907420.00</t>
+          <t>541620.00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1693,32 +1693,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CUST-010</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>270000.00</t>
+          <t>833000.00</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>48600.00</t>
+          <t>149940.00</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>318600.00</t>
+          <t>982940.00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1740,32 +1740,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CUST-010</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>890000.00</t>
+          <t>270000.00</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>160200.00</t>
+          <t>48600.00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>1050200.00</t>
+          <t>318600.00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1787,32 +1787,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>436000.00</t>
+          <t>807000.00</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>78480.00</t>
+          <t>145260.00</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>514480.00</t>
+          <t>952260.00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1933,27 +1933,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>833000.00</t>
+          <t>686000.00</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>149940.00</t>
+          <t>123480.00</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>982940.00</t>
+          <t>809480.00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CUST-004</t>
+          <t>CUST-005</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CUST-004</t>
+          <t>CUST-005</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CUST-006</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2131,17 +2131,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>116000.00</t>
+          <t>226000.00</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>20880.00</t>
+          <t>40680.00</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>136880.00</t>
+          <t>266680.00</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2163,32 +2163,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-011</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>271000.00</t>
+          <t>442000.00</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>48780.00</t>
+          <t>79560.00</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>319780.00</t>
+          <t>521560.00</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CUST-008</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2225,17 +2225,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>118000.00</t>
+          <t>797000.00</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>21240.00</t>
+          <t>143460.00</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>139240.00</t>
+          <t>940460.00</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CUST-004</t>
+          <t>CUST-005</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2272,17 +2272,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>277000.00</t>
+          <t>508000.00</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>49860.00</t>
+          <t>91440.00</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>326860.00</t>
+          <t>599440.00</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2304,32 +2304,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CUST-009</t>
+          <t>CUST-005</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>715000.00</t>
+          <t>85000.00</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>128700.00</t>
+          <t>15300.00</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>843700.00</t>
+          <t>100300.00</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CUST-009</t>
+          <t>CUST-011</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2445,32 +2445,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-011</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>573000.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>103140.00</t>
+          <t>79740.00</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>676140.00</t>
+          <t>522740.00</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2492,32 +2492,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CUST-006</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>746000.00</t>
+          <t>755000.00</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>134280.00</t>
+          <t>135900.00</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>880280.00</t>
+          <t>890900.00</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2544,27 +2544,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>256000.00</t>
+          <t>140000.00</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>46080.00</t>
+          <t>25200.00</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>302080.00</t>
+          <t>165200.00</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2586,32 +2586,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CUST-005</t>
+          <t>CUST-011</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>872000.00</t>
+          <t>781000.00</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>156960.00</t>
+          <t>140580.00</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>1028960.00</t>
+          <t>921580.00</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CUST-010</t>
+          <t>CUST-002</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2648,17 +2648,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>802000.00</t>
+          <t>823000.00</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>144360.00</t>
+          <t>148140.00</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>946360.00</t>
+          <t>971140.00</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2680,32 +2680,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>181000.00</t>
+          <t>83000.00</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>32580.00</t>
+          <t>14940.00</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>213580.00</t>
+          <t>97940.00</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2727,32 +2727,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CUST-001</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>657000.00</t>
+          <t>449000.00</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>118260.00</t>
+          <t>80820.00</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>775260.00</t>
+          <t>529820.00</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2774,32 +2774,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>547000.00</t>
+          <t>119000.00</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>98460.00</t>
+          <t>21420.00</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>645460.00</t>
+          <t>140420.00</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2821,32 +2821,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CUST-004</t>
+          <t>CUST-002</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>489000.00</t>
+          <t>537000.00</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>88020.00</t>
+          <t>96660.00</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>577020.00</t>
+          <t>633660.00</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2868,32 +2868,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CUST-002</t>
+          <t>CUST-003</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>178000.00</t>
+          <t>349000.00</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>32040.00</t>
+          <t>62820.00</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>210040.00</t>
+          <t>411820.00</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2915,32 +2915,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CUST-002</t>
+          <t>CUST-005</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>245000.00</t>
+          <t>748000.00</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>44100.00</t>
+          <t>134640.00</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>289100.00</t>
+          <t>882640.00</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2962,32 +2962,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CUST-006</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>753000.00</t>
+          <t>133000.00</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>135540.00</t>
+          <t>23940.00</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>888540.00</t>
+          <t>156940.00</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3009,32 +3009,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CUST-004</t>
+          <t>CUST-002</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>748000.00</t>
+          <t>605000.00</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>134640.00</t>
+          <t>108900.00</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>882640.00</t>
+          <t>713900.00</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3061,27 +3061,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>133000.00</t>
+          <t>222000.00</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>23940.00</t>
+          <t>39960.00</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>156940.00</t>
+          <t>261960.00</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3108,27 +3108,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>605000.00</t>
+          <t>149000.00</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>108900.00</t>
+          <t>26820.00</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>713900.00</t>
+          <t>175820.00</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3150,32 +3150,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CUST-005</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>222000.00</t>
+          <t>201000.00</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>39960.00</t>
+          <t>36180.00</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>261960.00</t>
+          <t>237180.00</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3197,32 +3197,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CUST-002</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>149000.00</t>
+          <t>699000.00</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>26820.00</t>
+          <t>125820.00</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>175820.00</t>
+          <t>824820.00</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3244,32 +3244,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CUST-001</t>
+          <t>CUST-010</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>201000.00</t>
+          <t>244000.00</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>36180.00</t>
+          <t>43920.00</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>237180.00</t>
+          <t>287920.00</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3291,32 +3291,32 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-003</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>699000.00</t>
+          <t>545000.00</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>125820.00</t>
+          <t>98100.00</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>824820.00</t>
+          <t>643100.00</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3338,32 +3338,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>551000.00</t>
+          <t>760000.00</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>99180.00</t>
+          <t>136800.00</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>650180.00</t>
+          <t>896800.00</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3385,32 +3385,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CUST-009</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>744000.00</t>
+          <t>476000.00</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>133920.00</t>
+          <t>85680.00</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>877920.00</t>
+          <t>561680.00</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3432,32 +3432,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CUST-008</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>463000.00</t>
+          <t>798000.00</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>83340.00</t>
+          <t>143640.00</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>546340.00</t>
+          <t>941640.00</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3479,32 +3479,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CUST-011</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>615000.00</t>
+          <t>98000.00</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>110700.00</t>
+          <t>17640.00</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>725700.00</t>
+          <t>115640.00</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3526,32 +3526,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-003</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>841000.00</t>
+          <t>217000.00</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>151380.00</t>
+          <t>39060.00</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>992380.00</t>
+          <t>256060.00</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3573,32 +3573,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-008</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>464000.00</t>
+          <t>471000.00</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>83520.00</t>
+          <t>84780.00</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>547520.00</t>
+          <t>555780.00</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3620,32 +3620,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CUST-001</t>
+          <t>CUST-007</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>218000.00</t>
+          <t>402000.00</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>39240.00</t>
+          <t>72360.00</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>257240.00</t>
+          <t>474360.00</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3667,32 +3667,32 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CUST-012</t>
+          <t>CUST-002</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>69000.00</t>
+          <t>641000.00</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>12420.00</t>
+          <t>115380.00</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>81420.00</t>
+          <t>756380.00</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CUST-007</t>
+          <t>CUST-001</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3729,17 +3729,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>69000.00</t>
+          <t>641000.00</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>12420.00</t>
+          <t>115380.00</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>81420.00</t>
+          <t>756380.00</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">

</xml_diff>